<commit_message>
Update remove item in cartpagetest
</commit_message>
<xml_diff>
--- a/data/test-data.xlsx
+++ b/data/test-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\duypt\IdeaProjects\Selenium-testing-portfolio\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E063FE0D-0182-418D-ABA8-DFF5AD98B5B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45F42FE8-2A72-4B9E-8A7C-7CAE29DE16BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{28160BE1-BB2E-4917-B570-2D11B4AEE20B}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{28160BE1-BB2E-4917-B570-2D11B4AEE20B}"/>
   </bookViews>
   <sheets>
     <sheet name="loginPageTest" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="44">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Cart Badge</t>
   </si>
   <si>
-    <t>2, 5</t>
-  </si>
-  <si>
     <t>Total amount</t>
   </si>
   <si>
@@ -156,6 +153,24 @@
   </si>
   <si>
     <t>Checkout success</t>
+  </si>
+  <si>
+    <t>action</t>
+  </si>
+  <si>
+    <t>add</t>
+  </si>
+  <si>
+    <t>Sauce Labs Fleece Jacket, Sauce Labs Bolt T-Shirt</t>
+  </si>
+  <si>
+    <t>remove</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bike Light, Sauce Labs Onesie</t>
   </si>
 </sst>
 </file>
@@ -229,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -239,6 +254,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -711,7 +727,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -730,8 +746,8 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
+      <c r="B2" t="s">
+        <v>42</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -741,8 +757,8 @@
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
-        <v>25</v>
+      <c r="B3" s="9" t="s">
+        <v>43</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -757,44 +773,67 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FA77806-C650-45EC-9A76-042EE8F211F3}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" customWidth="1"/>
     <col min="2" max="2" width="45.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3">
         <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -822,16 +861,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>32</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>13</v>
@@ -842,17 +881,17 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D2" s="8"/>
       <c r="E2" s="8">
         <v>123</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -860,17 +899,17 @@
         <v>5</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3" s="8">
         <v>123</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -878,17 +917,17 @@
         <v>6</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4" s="8"/>
       <c r="F4" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -896,19 +935,19 @@
         <v>7</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" s="8">
         <v>123</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>